<commit_message>
chuẩn bị demo 1
</commit_message>
<xml_diff>
--- a/DATA_TEST_CASE4_LIEN_MIEN_1_DON.xlsx
+++ b/DATA_TEST_CASE4_LIEN_MIEN_1_DON.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 4 - Don Lien Mien (1 Don)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case 4 - Don Lien Mien (2 Don)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DanhMucHanhChinh" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
     <col width="66" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="64" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
@@ -801,6 +801,126 @@
       <c r="Z2" s="5" t="inlineStr">
         <is>
           <t>Giao giờ hành chính tại Phòng Đào tạo PTIT Hà Nội</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Đặc sản Miền Trung</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>0904000004</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Số 24 Đường Nguyễn Văn Linh</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Phường Nam Dương</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Thành phố Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Trần Thị Bích Ngọc</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Học viện Công nghệ Bưu chính Viễn thông, Km 10 Trần Phú, Mộ Lao</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Phường Hà Đông</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Thành phố Hà Nội</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Set đặc sản Miền Trung (Bánh khô mè, Mực rim me, Trà Sâm Dứa)</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>800000</v>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Thường</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>STANDARD (Tiêu chuẩn)</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>PICKUP (Shipper lấy tận nơi)</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>Hôm nay</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>Ca Sáng (08:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>SENDER (Người gửi trả)</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>COD (Thu hộ COD)</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>Giao giờ hành chính tại Hà Đông</t>
         </is>
       </c>
     </row>

</xml_diff>